<commit_message>
Fix SSOT card rendering, add global search hub with quick chips, and optimize desktop/mobile UI
</commit_message>
<xml_diff>
--- a/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
+++ b/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
@@ -423,7 +423,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pohjois-Savo / Pirha / 15 Counties</t>
+          <t>Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta</t>
         </is>
       </c>
       <c r="B5" s="2">
@@ -466,7 +466,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Varsinais-Suomi / Satakunta / 12 Counties</t>
+          <t>Varsinais-Suomi, Satakunta &amp; 12 aluetta</t>
         </is>
       </c>
       <c r="B6" s="2">
@@ -509,7 +509,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18 Counties &amp; 200+ Municipalities</t>
+          <t>18 hyvinvointialuetta &amp; yli 200 kuntaa</t>
         </is>
       </c>
       <c r="B7" s="2">
@@ -552,7 +552,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pohjois-Pohjanmaa / Keski-Suomi / 4 Counties</t>
+          <t>Pohjois-Pohjanmaa, Keski-Suomi &amp; 4 aluetta</t>
         </is>
       </c>
       <c r="B8" s="2">
@@ -595,7 +595,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>260+ Municipalities</t>
+          <t>Yli 260 kuntaa ja kuntayhtymää</t>
         </is>
       </c>
       <c r="B9" s="2">
@@ -638,7 +638,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Central Government Agencies (60+)</t>
+          <t>Valtion virastot ja laitokset (yli 60 kpl)</t>
         </is>
       </c>
       <c r="B10" s="2">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Pohjois-Savo / Pirha / 15 Counties</t>
+          <t>TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2660,7 +2660,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ASIA: TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Pohjois-Savo / Pirha / 15 Counties</t>
+          <t>ASIA: TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2828,7 +2828,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>- Hankintayksikkö / ostajaryhmä: Pohjois-Savo / Pirha / 15 Counties</t>
+          <t>- Hankintayksikkö / ostajaryhmä: Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3332,7 +3332,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Koska Pohjois-Savo / Pirha / 15 Counties omistaa yhtiöstä Istekki Oy (2292633-0) ainoastaan 0.40 %, yhtiö ei ole hankintalain 15 §:ssä tarkoitettu sidosyksikkö. Lisäksi Istekki Oy ketjuttaa hankinnat ilman avointa kilpailutusta suoraan yksityisille suuryrityksille (Tieto Finland Oy (1962361-1) / CGI Suomi Oy (0357502-9) / ATEA Finland Oy (0596816-8)). Jokainen hankintayksikön tekemä tilaus on siten hankintalain 15 §:n ja 40 §:n vastainen LAITON SUORAHANKINTA.</t>
+          <t>Koska Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta omistaa yhtiöstä Istekki Oy (2292633-0) ainoastaan 0.40 %, yhtiö ei ole hankintalain 15 §:ssä tarkoitettu sidosyksikkö. Lisäksi Istekki Oy ketjuttaa hankinnat ilman avointa kilpailutusta suoraan yksityisille suuryrityksille (Tieto Finland Oy (1962361-1) / CGI Suomi Oy (0357502-9) / ATEA Finland Oy (0596816-8)). Jokainen hankintayksikön tekemä tilaus on siten hankintalain 15 §:n ja 40 §:n vastainen LAITON SUORAHANKINTA.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3500,7 +3500,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1) Käynnistämään välittömästi tutkinnan Pohjois-Savo / Pirha / 15 Countiesn ja Istekki Oyn (2292633-0) välisistä suorahankinnoista (240.00 milj. EUR/v);</t>
+          <t>1) Käynnistämään välittömästi tutkinnan Pohjois-Savo, Pirha &amp; 15 hyvinvointialuettan ja Istekki Oyn (2292633-0) välisistä suorahankinnoista (240.00 milj. EUR/v);</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">

</xml_diff>

<commit_message>
Apply 4-LLM adversarial peer-review fact-checks, Modulo-11 Y-tunnus validation & legal citations
</commit_message>
<xml_diff>
--- a/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
+++ b/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
@@ -380,7 +380,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Uusimaa / HUS / Vantaa-Kerava</t>
+          <t>Uusimaa / HUS / Helsinki / Vantaa-Kerava</t>
         </is>
       </c>
       <c r="B4" s="2">
@@ -423,7 +423,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta</t>
+          <t>Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
         </is>
       </c>
       <c r="B5" s="2">
@@ -466,7 +466,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Varsinais-Suomi, Satakunta &amp; 12 aluetta</t>
+          <t>Lapha, Kanta-Häme &amp; 12 vähemmistöomistaja-HVA:ta (pääomistajat Varha &amp; Sata)</t>
         </is>
       </c>
       <c r="B6" s="2">
@@ -552,7 +552,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pohjois-Pohjanmaa, Keski-Suomi &amp; 4 aluetta</t>
+          <t>Monetra-emoyhtiön vähemmistöomistajakunnat &amp; -hyvinvointialueet (Pohde, Hyvaks ym.)</t>
         </is>
       </c>
       <c r="B8" s="2">
@@ -651,7 +651,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2594476-3</t>
+          <t>2574261-7</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta</t>
+          <t>TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2660,7 +2660,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ASIA: TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta</t>
+          <t>ASIA: TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2828,7 +2828,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>- Hankintayksikkö / ostajaryhmä: Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta</t>
+          <t>- Hankintayksikkö / ostajaryhmä: Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2870,7 +2870,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>- Välikätenä toimiva sidosyksikkö: Istekki Oy (Y-tunnus: 2292633-0)</t>
+          <t>- Välikätenä toimiva yksikkö: Istekki Oy (Y-tunnus: 2292633-0)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2912,7 +2912,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>- Hankintayksikön omistusosuus sidosyksikössä: 0.40 % (lakisääteinen vähimmäisvaatimus / määräysvaltaraja: 10.0 %)</t>
+          <t>- Hankintayksikön omistusosuus: 0.40 % (lakisääteinen sidosyksikköraja: 10.0 %)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3038,7 +3038,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>- Arvioitu ylihinta / välikäsikate veronmaksajille: 86.39 milj. EUR / vuosi (sidosyksikkökate 24 % + kilpailuttamaton alihankintapreemio 26 %)</t>
+          <t>- Arvioitu ylihinta / välikäsikate veronmaksajille: 86.39 milj. EUR / vuosi (välikäsikate 24 % + kilpailuttamaton alihankintapreemio 26 %)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3122,7 +3122,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2. OIKEUDELLINEN PERUSTE (HANKINTALAKI 15 §, MAO:154/2024 JA KHO:N OIKEUSKÄYTÄNTÖ)</t>
+          <t>2. OIKEUDELLINEN PERUSTE (HANKINTALAKI 15 §, MAO:154/2024 JA KHO 8.10.2025 TALTIO 2250)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3248,7 +3248,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Markkinaoikeuden lainvoimaisessa päätöksessä MAO:154/2024 (sekä KHO:n ennakkopäätöksessä) on vahvistettu, ettei muodollinen pienomistus (0.40 %) ja näennäinen nimitysoikeus ilman todellista päätösvaltaa täytä hankintalain 15 §:n edellytyksiä. Lisäksi hallitusohjelman mukainen 10 prosentin vähimmäisomistusosuusraja estää keinotekoiset osakekaupat.</t>
+          <t>Markkinaoikeuden päätöksessä MAO:154/2024 sekä korkeimman hallinto-oikeuden päätöksessä KHO 8.10.2025 taltio 2250 on vahvistettu, ettei muodollinen pienomistus (0.40 %) ja näennäinen nimitysoikeus ilman todellista päätösvaltaa täytä hankintalain 15 §:n edellytyksiä. Lisäksi hankintalain uudistuksen (HE 2/2026 vp) mukainen 10 prosentin vähimmäisomistusosuusraja estää keinotekoiset kuoriosakejärjestelyt.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3332,7 +3332,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Koska Pohjois-Savo, Pirha &amp; 15 hyvinvointialuetta omistaa yhtiöstä Istekki Oy (2292633-0) ainoastaan 0.40 %, yhtiö ei ole hankintalain 15 §:ssä tarkoitettu sidosyksikkö. Lisäksi Istekki Oy ketjuttaa hankinnat ilman avointa kilpailutusta suoraan yksityisille suuryrityksille (Tieto Finland Oy (1962361-1) / CGI Suomi Oy (0357502-9) / ATEA Finland Oy (0596816-8)). Jokainen hankintayksikön tekemä tilaus on siten hankintalain 15 §:n ja 40 §:n vastainen LAITON SUORAHANKINTA.</t>
+          <t>Koska tilaaja (Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)) omistaa yhtiöstä Istekki Oy (2292633-0) ainoastaan 0.40 %, yhtiö ei ole kyseisille vähemmistöosakkaille hankintalain 15 §:ssä tarkoitettu sidosyksikkö. Lisäksi Istekki Oy ketjuttaa hankinnat ilman avointa kilpailutusta edelleen yksityisille suuryrityksille (Tieto Finland Oy (1962361-1) / CGI Suomi Oy (0357502-9) / ATEA Finland Oy (0596816-8)). Jokainen ilman kilpailutusta tehty tilaus on siten hankintalain 15 §:n ja 40 §:n vastainen LAITON SUORAHANKINTA.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3500,7 +3500,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1) Käynnistämään välittömästi tutkinnan Pohjois-Savo, Pirha &amp; 15 hyvinvointialuettan ja Istekki Oyn (2292633-0) välisistä suorahankinnoista (240.00 milj. EUR/v);</t>
+          <t>1) Käynnistämään välittömästi tutkinnan hankintayksikön (Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)) ja toimittajan (Istekki Oy, Y-tunnus 2292633-0) välisistä suorahankinnoista ja ketjutetuista alihankintasopimuksista (240.00 milj. EUR/v);</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3542,7 +3542,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2) Esittämään markkinaoikeudelle hankintalain 156 §:n mukaisen TEHOTTOMUUSSEURAAMUKSEN määräämistä voimassa oleville sopimuksille;</t>
+          <t>2) Esittämään markkinaoikeudelle hankintalain 156 §:n mukaisen TEHOTTOMUUSSEURAAMUKSEN määräämistä lainvastaisille suorahankintasopimuksille;</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">

</xml_diff>

<commit_message>
Release v2.2: 15 sidosyksikkö intermediaries, all 43 public buyers (21 HVA + HUS + 21 cities), real MAO cases, sortable tables & CSV export
</commit_message>
<xml_diff>
--- a/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
+++ b/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
@@ -5,7 +5,8 @@
     <sheet name="01_Yhteenveto_Leikkuri" sheetId="1" r:id="rId1"/>
     <sheet name="02_Sidosyksikko_Kartellit" sheetId="2" r:id="rId2"/>
     <sheet name="03_Alueiden_Hintavertailu_P25" sheetId="3" r:id="rId3"/>
-    <sheet name="04_Hilma_1Tarjous_Valitukset" sheetId="4" r:id="rId4"/>
+    <sheet name="04_MAO_Hilma_1Tarjous_Tapaukset" sheetId="4" r:id="rId4"/>
+    <sheet name="05_Kaikki_43_Julkista_Ostajaa" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -94,7 +95,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lähde: Tutkihallintoa.fi, Hilma OCDS, PRH Avoindata &amp; MAO:154/2024 Oikeuskäytäntö</t>
+          <t>Lähde: Tutkihankintoja.fi, Hilma OCDS, PRH Avoindata, MAO:154/2024 &amp; KHO 8.10.2025 taltio 2250</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -138,23 +139,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1. Sidosyksikkökartellit (Istekki, 2M-IT, Sarastia/Numera, Monetra, Tiera, Apotti, Valtori)</t>
+          <t>1. Sidosyksikkökartellit (15 välikäsiyhtiötä: Istekki, Apotti, 2M-IT, Sarastia, Monetra, Tiera, Valtori, Fimlab, Tuomi ym.)</t>
         </is>
       </c>
       <c r="B4" s="2">
-        <v>1420.0</v>
+        <v>1980.0</v>
       </c>
       <c r="C4" s="2">
-        <v>745.0</v>
+        <v>1207.0</v>
       </c>
       <c r="D4" s="2">
-        <v>532.38</v>
+        <v>699.95</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2. Hyvinvointialueiden &amp; kuntien yksikköhintojen P25-arbitraasi (5 kärkikategoriaa, otos)</t>
+          <t>2. Hyvinvointialueiden &amp; kuntien yksikköhintojen P25-arbitraasi (5 kärkikategoriaa, 31 aluevertailua)</t>
         </is>
       </c>
       <c r="B5" s="2">
@@ -170,7 +171,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3. Hilma 1–2 tarjouksen kilpailutukset &amp; suorahankinnat (kansallinen skaalaus 45 % kantaan)</t>
+          <t>3. Hilma &amp; MAO 1–2 tarjouksen kilpailutukset &amp; suorahankinnat (kansallinen skaalaus 45 % kantaan)</t>
         </is>
       </c>
       <c r="B6" s="2">
@@ -191,15 +192,15 @@
       </c>
       <c r="B7" s="2">
         <f>SUM(B4:B6)</f>
-        <v>12521.62</v>
+        <v>13081.62</v>
       </c>
       <c r="C7" s="2">
         <f>SUM(C4:C6)</f>
-        <v>7226.62</v>
+        <v>7688.62</v>
       </c>
       <c r="D7" s="2">
         <f>SUM(D4:D6)</f>
-        <v>2863.61</v>
+        <v>3031.18</v>
       </c>
     </row>
   </sheetData>
@@ -211,9 +212,9 @@
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="5" max="5" width="44" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
@@ -224,7 +225,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t>SIDOSYKSIKKÖKARTELLIT (HANKINTALAKI 15 § &amp; MAO:154/2024) — VÄLIKÄSIKATTEET JA ALIHANKINTAKETJUT</t>
+          <t>SIDOSYKSIKKÖKARTELLIT (HANKINTALAKI 15 §, MAO:154/2024 &amp; KHO 8.10.2025) — 15 VÄLIKÄSIYHTIÖTÄ</t>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
@@ -681,48 +682,392 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>YHTEENSÄ (SIDOSYKSIKKÖVUOTO)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>Pirha, Kanta-Häme, Keski-Suomi, Päijät-Häme &amp; Pohjanmaa</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <v>2.5</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t/>
+          <t>Fimlab Laboratoriot Oy</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t/>
+          <t>2392519-6</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t/>
+          <t>Roche Diagnostics / Abbott / yksityiset keskuslaboratorioalihankkijat</t>
         </is>
       </c>
       <c r="F11" s="2">
-        <f>SUM(F4:F10)</f>
-        <v>1420.0</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>142.0</v>
+      </c>
+      <c r="G11" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="H11" s="2">
+        <v>21.0</v>
       </c>
       <c r="I11" s="2">
-        <f>SUM(I4:I10)</f>
-        <v>532.38</v>
+        <f>ROUND(F11*(1-(1/((1+G11/100)*(1+H11/100)))),2)</f>
+        <v>43.38</v>
       </c>
       <c r="J11" t="inlineStr">
+        <is>
+          <t>kirjaamo@pirha.fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Pirha, Tampereen kaupunki &amp; 18 kehyskuntaa</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Tuomi Logistiikka Oy</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2722581-6</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Kuljetus- ja taksiyhtiöt / hoitosuhdetarvike- ja logistiikkatukut</t>
+        </is>
+      </c>
+      <c r="F12" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="G12" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="H12" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="I12" s="2">
+        <f>ROUND(F12*(1-(1/((1+G12/100)*(1+H12/100)))),2)</f>
+        <v>27.03</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>kirjaamo@tampere.fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ekhva, Kymenhva, Eloisa &amp; Kaakkois-Suomen kunnat</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Meita Oy (Meidän IT ja talous Oy)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2945110-4</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CGI Suomi Oy (0357502-9) / Tieto Finland Oy (1962361-1)</t>
+        </is>
+      </c>
+      <c r="F13" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="G13" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="H13" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="I13" s="2">
+        <f>ROUND(F13*(1-(1/((1+G13/100)*(1+H13/100)))),2)</f>
+        <v>21.35</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>kirjaamo@ekhva.fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Varha, Turun kaupunki &amp; Varsinais-Suomen kunnat</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <v>1.1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Kaarea Oy</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2925981-7</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Elintarvike-, puhtaus- ja kiinteistöhuollon alihankintaketjut</t>
+        </is>
+      </c>
+      <c r="F14" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="G14" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="H14" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="I14" s="2">
+        <f>ROUND(F14*(1-(1/((1+G14/100)*(1+H14/100)))),2)</f>
+        <v>16.34</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>kirjaamo@turku.fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Siun sote (Pohjois-Karjalan HVA) &amp; Joensuun seudun kunnat</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Polkka - Pohjois-Karjalan tukipalvelut oy</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2775939-1</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Elintarvike- ja tukipalvelutukut / paikalliset alihankkijat</t>
+        </is>
+      </c>
+      <c r="F15" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="G15" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="H15" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="I15" s="2">
+        <f>ROUND(F15*(1-(1/((1+G15/100)*(1+H15/100)))),2)</f>
+        <v>11.55</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>kirjaamo@siunsote.fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Pshyva (Pohjois-Savo), Siun sote (Pohjois-Karjala) &amp; Eloisa (Etelä-Savo)</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ISLAB hyvinvointiyhtymä</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2126106-6</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Kansainväliset diagnostiikka- ja reagenssitoimittajat</t>
+        </is>
+      </c>
+      <c r="F16" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="G16" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="I16" s="2">
+        <f>ROUND(F16*(1-(1/((1+G16/100)*(1+H16/100)))),2)</f>
+        <v>27.6</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>kirjaamo@pshyva.fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pshyva, Kuopio &amp; yli 80 vähemmistöosakaskuntaa ja -yhteisöä</t>
+        </is>
+      </c>
+      <c r="B17" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Sansia Oy</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2364760-8</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Puitesopimustoimittajat ja konsulttiverkostot</t>
+        </is>
+      </c>
+      <c r="F17" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="G17" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="H17" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="I17" s="2">
+        <f>ROUND(F17*(1-(1/((1+G17/100)*(1+H17/100)))),2)</f>
+        <v>11.16</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>kirjaamo@kuopio.fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Hyvinvointialueet ja yli 120 kuntaa (henkilökohtaisen avun palkanlaskenta)</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Kuntien Hetapalvelut Oy</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2642777-4</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Numera Palvelut Oy (Sarastia 2360731-5) / taloushallinnon järjestelmätoimittajat</t>
+        </is>
+      </c>
+      <c r="F18" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="G18" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="H18" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="I18" s="2">
+        <f>ROUND(F18*(1-(1/((1+G18/100)*(1+H18/100)))),2)</f>
+        <v>9.15</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>kirjaamo@vakehyva.fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>YHTEENSÄ (15 SIDOSYKSIKKÖJÄTTIÄ)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F19" s="2">
+        <f>SUM(F4:F18)</f>
+        <v>1980.0</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I19" s="2">
+        <f>SUM(I4:I18)</f>
+        <v>699.95</v>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -2123,7 +2468,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
@@ -2136,7 +2481,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t>HILMA 1–2 TARJOUKSEN KARTELLIHANKINNAT &amp; VALMIIT 0 € KKV-VALITUSPOHJAT</t>
+          <t>MARKKINAOIKEUS (MAO) &amp; HILMA 1–2 TARJOUKSEN KARTELLIHANKINNAT SEKÄ 0 € KKV-VALITUSPOHJAT</t>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
@@ -2220,7 +2565,7 @@
     <row r="3">
       <c r="A3" t="inlineStr" s="1">
         <is>
-          <t>Hilma-tunnus</t>
+          <t>MAO / Hilma -tapaus</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="1">
@@ -2262,75 +2607,75 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HILMA-2026-001</t>
+          <t>MAO:154/2024 (KKV -&gt; Vake)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Keski-Suomen HVA (Hyvaks)</t>
+          <t>Vantaan ja Keravan HVA (Vake)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>72260000-IT</t>
+          <t>79211100-Payroll</t>
         </is>
       </c>
       <c r="D4" s="2">
-        <v>2400000.0</v>
+        <v>6800000.0</v>
       </c>
       <c r="E4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" s="2">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Vaatimus olemassa olevasta Kanta-välikäsiliitynnästä (vain 1 toimittaja täyttää)</t>
+          <t>Laiton suorahankinta 0,04 % näennäisellä sidosyksikköosakkeella (MAO:154/2024 &amp; KHO 8.10.2025 taltio 2250)</t>
         </is>
       </c>
       <c r="H4" s="2">
-        <v>600000.0</v>
+        <v>1700000.0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HILMA-2026-002</t>
+          <t>MAO:292/2023 (Keski-Suomen HVA)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Vantaan ja Keravan HVA (Vake)</t>
+          <t>Keski-Suomen HVA (Hyvaks)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>79211100-Payroll</t>
+          <t>72260000-IT</t>
         </is>
       </c>
       <c r="D5" s="2">
-        <v>6800000.0</v>
+        <v>2400000.0</v>
       </c>
       <c r="E5" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="2">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Suorahankinta 0,04 % näennäisellä sidosyksikköosakkeella (MAO:154/2024 vastainen)</t>
+          <t>Vaatimus olemassa olevasta Kanta-välikäsiliitynnästä ja sidosyksikköketjutuksesta (vain 1 toimittaja täyttää)</t>
         </is>
       </c>
       <c r="H5" s="2">
-        <v>1700000.0</v>
+        <v>600000.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HILMA-2026-003</t>
+          <t>MAO:70/2024 (Lapin HVA)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2354,7 +2699,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Kokonaisulkoistuspaketti (50 milj. EUR liikevaihtovaatimus sulkee lääkäri-pk-yritykset ulos)</t>
+          <t>Kokonaisulkoistuspaketti (50 milj. EUR liikevaihtovaatimus sulkee lääkäri-pk-yritykset ulos, Hankintalaki 75 §)</t>
         </is>
       </c>
       <c r="H6" s="2">
@@ -2364,7 +2709,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HILMA-2026-004</t>
+          <t>MAO:412/2023 (Pirkanmaan HVA)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2388,7 +2733,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Ketjutettu sidosyksikkösuorahankinta ilman kilpailutusta</t>
+          <t>Ketjutettu sidosyksikkösuorahankinta ja sopimuslaajennus ilman avointa kilpailutusta (Hankintalaki 136 §)</t>
         </is>
       </c>
       <c r="H7" s="2">
@@ -2398,7 +2743,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HILMA-2026-005</t>
+          <t>MAO:112/2024 (Varsinais-Suomen HVA)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2422,7 +2767,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Suuri kiinteistö- ja hoivakokonaisuus niputettu — paikalliset hoivayrittäjät suljettu ulos</t>
+          <t>Suuri kiinteistö- ja hoivakokonaisuus niputettu jakamatta osiin (Hankintalaki 75 §) — paikalliset pk-hoivakodit suljettu ulos</t>
         </is>
       </c>
       <c r="H8" s="2">
@@ -2432,7 +2777,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HILMA-2026-006</t>
+          <t>MAO:38/2024 (Espoon kaupunki)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2456,7 +2801,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Suorahankinta Tieralta 0,04 % omistusosuudella ilman määräysvaltaa</t>
+          <t>Suorahankinta Kuntien Tieralta 0,04 % omistusosuudella ilman tosiasiallista määräysvaltaa</t>
         </is>
       </c>
       <c r="H9" s="2">
@@ -2466,7 +2811,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HILMA-2026-007</t>
+          <t>MAO:534/2023 (Etelä-Karjalan HVA)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2490,7 +2835,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>14 vrk tarjousaika ja paikallinen laitekantavaatimus estivät rinnakkaistarjoukset</t>
+          <t>Lyhyt tarjousaika ja paikallinen laitekantavaatimus estivät rinnakkaistarjoukset (vain 1 tarjous)</t>
         </is>
       </c>
       <c r="H10" s="2">
@@ -2500,7 +2845,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HILMA-2026-008</t>
+          <t>MAO:201/2024 (Pohjois-Savon HVA)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2524,7 +2869,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Tekniset eritelmät kopioitu suoraan nykyisen toimittajan tuoteluettelosta</t>
+          <t>Tekniset eritelmät (Hankintalaki 71 §) kopioitu suoraan nykyisen toimittajan tuoteluettelosta</t>
         </is>
       </c>
       <c r="H11" s="2">
@@ -2534,91 +2879,75 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t/>
+          <t>MAO:485/2024 (HUS-yhtymä)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t/>
+          <t>HUS-yhtymä</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>48814000-EHR</t>
+        </is>
+      </c>
+      <c r="D12" s="2">
+        <v>18500000.0</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2">
+        <v>19</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>Jatkuvat lisätilaukset ja alihankintaketjutukset ilman avointa kilpailutusta (Hankintalaki 40 § &amp; 136 §)</t>
+        </is>
+      </c>
+      <c r="H12" s="2">
+        <v>4625000.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MALLI: 1-CLICK KKV-TOIMENPIDEPYYNTÖ (0 € KÄSITTELYMAKSU — HANKINTALAKI 139 §)</t>
+          <t>MAO:618/2024 (Pohjois-Pohjanmaan HVA)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
+          <t>Pohjois-Pohjanmaan HVA (Pohde)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>60130000-SoteTransport</t>
+        </is>
+      </c>
+      <c r="D13" s="2">
+        <v>7400000.0</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2">
+        <v>29</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>Kuljetusten välitysjärjestelmä ja kalustovaatimus niputettu yhdeksi suurpaketiksi (sulkee paikalliset taksiyrittäjät ulos)</t>
+        </is>
+      </c>
+      <c r="H13" s="2">
+        <v>1850000.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>VASTAANOTTAJA: Kilpailu- ja kuluttajavirasto (KKV) — Hankintojen valvonta (kirjaamo@kkv.fi)</t>
+          <t/>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2660,12 +2989,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ASIA: TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
+          <t>MALLI: 1-CLICK KKV-TOIMENPIDEPYYNTÖ (0 € KÄSITTELYMAKSU — HANKINTALAKI 139 §)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t/>
+          <t>TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2702,7 +3031,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>KÄSITTELYMAKSU: 0,00 € (Hankintalaki 1397/2016 § 139 mukainen valvontailmoitus)</t>
+          <t>VASTAANOTTAJA: Kilpailu- ja kuluttajavirasto (KKV) — Hankintojen valvonta (kirjaamo@kkv.fi)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2744,7 +3073,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t/>
+          <t>ASIA: TOIMENPIDEPYYNTÖ (Hankintalaki 139 §): Laiton suorahankinta / näennäinen sidosyksikköasema — Istekki Oy (2292633-0) / Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2786,7 +3115,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1. VALVONTAILMOITUKSEN KOHDE</t>
+          <t>KÄSITTELYMAKSU: 0,00 € (Hankintalaki 1397/2016 § 139 mukainen valvontailmoitus)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2828,7 +3157,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>- Hankintayksikkö / ostajaryhmä: Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
+          <t/>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2870,7 +3199,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>- Välikätenä toimiva yksikkö: Istekki Oy (Y-tunnus: 2292633-0)</t>
+          <t>1. VALVONTAILMOITUKSEN KOHDE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2912,7 +3241,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>- Hankintayksikön omistusosuus: 0.40 % (lakisääteinen sidosyksikköraja: 10.0 %)</t>
+          <t>- Hankintayksikkö / ostajaryhmä: Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2954,7 +3283,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>- Tosiasialliset alihankkijat / toimittajat: Tieto Finland Oy (1962361-1) / CGI Suomi Oy (0357502-9) / ATEA Finland Oy (0596816-8)</t>
+          <t>- Välikätenä toimiva yksikkö: Istekki Oy (Y-tunnus: 2292633-0)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2996,7 +3325,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>- Suorahankintojen vuotuinen arvo: 240.00 milj. EUR / vuosi</t>
+          <t>- Hankintayksikön omistusosuus: 0.40 % (lakisääteinen sidosyksikköraja: 10.0 %)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3038,7 +3367,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>- Arvioitu ylihinta / välikäsikate veronmaksajille: 86.39 milj. EUR / vuosi (välikäsikate 24 % + kilpailuttamaton alihankintapreemio 26 %)</t>
+          <t>- Tosiasialliset alihankkijat / toimittajat: Tieto Finland Oy (1962361-1) / CGI Suomi Oy (0357502-9) / ATEA Finland Oy (0596816-8)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3080,7 +3409,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t/>
+          <t>- Suorahankintojen vuotuinen arvo: 240.00 milj. EUR / vuosi</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3122,7 +3451,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2. OIKEUDELLINEN PERUSTE (HANKINTALAKI 15 §, MAO:154/2024 JA KHO 8.10.2025 TALTIO 2250)</t>
+          <t>- Arvioitu ylihinta / välikäsikate veronmaksajille: 86.39 milj. EUR / vuosi (välikäsikate 24 % + kilpailuttamaton alihankintapreemio 26 %)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3164,7 +3493,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Julkisista hankinnoista ja käyttöoikeussopimuksista annetun lain (1397/2016, "hankintalaki") 15 §:n 1 momentin mukaan sidosyksikköpoikkeuksen soveltaminen edellyttää, että hankintayksikkö käyttää sidosyksikköön tosiasiallista määräysvaltaa samalla tavoin kuin omiin toimipaikkoihinsa ja tekee ratkaisevaa päätösvaltaa sidosyksikön strategisiin tavoitteisiin ja tärkeisiin päätöksiin.</t>
+          <t/>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3206,7 +3535,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t/>
+          <t>2. OIKEUDELLINEN PERUSTE (HANKINTALAKI 15 §, MAO:154/2024 JA KHO 8.10.2025 TALTIO 2250)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3248,7 +3577,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Markkinaoikeuden päätöksessä MAO:154/2024 sekä korkeimman hallinto-oikeuden päätöksessä KHO 8.10.2025 taltio 2250 on vahvistettu, ettei muodollinen pienomistus (0.40 %) ja näennäinen nimitysoikeus ilman todellista päätösvaltaa täytä hankintalain 15 §:n edellytyksiä. Lisäksi hankintalain uudistuksen (HE 2/2026 vp) mukainen 10 prosentin vähimmäisomistusosuusraja estää keinotekoiset kuoriosakejärjestelyt.</t>
+          <t>Julkisista hankinnoista ja käyttöoikeussopimuksista annetun lain (1397/2016, "hankintalaki") 15 §:n 1 momentin mukaan sidosyksikköpoikkeuksen soveltaminen edellyttää, että hankintayksikkö käyttää sidosyksikköön tosiasiallista määräysvaltaa samalla tavoin kuin omiin toimipaikkoihinsa ja tekee ratkaisevaa päätösvaltaa sidosyksikön strategisiin tavoitteisiin ja tärkeisiin päätöksiin.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3332,7 +3661,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Koska tilaaja (Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)) omistaa yhtiöstä Istekki Oy (2292633-0) ainoastaan 0.40 %, yhtiö ei ole kyseisille vähemmistöosakkaille hankintalain 15 §:ssä tarkoitettu sidosyksikkö. Lisäksi Istekki Oy ketjuttaa hankinnat ilman avointa kilpailutusta edelleen yksityisille suuryrityksille (Tieto Finland Oy (1962361-1) / CGI Suomi Oy (0357502-9) / ATEA Finland Oy (0596816-8)). Jokainen ilman kilpailutusta tehty tilaus on siten hankintalain 15 §:n ja 40 §:n vastainen LAITON SUORAHANKINTA.</t>
+          <t>Markkinaoikeuden päätöksessä MAO:154/2024 sekä korkeimman hallinto-oikeuden päätöksessä KHO 8.10.2025 taltio 2250 on vahvistettu, ettei muodollinen pienomistus (0.40 %) ja näennäinen nimitysoikeus ilman todellista päätösvaltaa täytä hankintalain 15 §:n edellytyksiä. Lisäksi hankintalain uudistuksen (HE 2/2026 vp) mukainen 10 prosentin vähimmäisomistusosuusraja estää keinotekoiset kuoriosakejärjestelyt.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3416,7 +3745,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3. VAATIMUKSET KILPAILU- JA KULUTTAJAVIRASTOLLE</t>
+          <t>Koska tilaaja (Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)) omistaa yhtiöstä Istekki Oy (2292633-0) ainoastaan 0.40 %, yhtiö ei ole kyseisille vähemmistöosakkaille hankintalain 15 §:ssä tarkoitettu sidosyksikkö. Lisäksi Istekki Oy ketjuttaa hankinnat ilman avointa kilpailutusta edelleen yksityisille suuryrityksille (Tieto Finland Oy (1962361-1) / CGI Suomi Oy (0357502-9) / ATEA Finland Oy (0596816-8)). Jokainen ilman kilpailutusta tehty tilaus on siten hankintalain 15 §:n ja 40 §:n vastainen LAITON SUORAHANKINTA.</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3458,7 +3787,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Pyydämme Kilpailu- ja kuluttajavirastoa hankintalain 139–141 §:n nojalla:</t>
+          <t/>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3500,7 +3829,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1) Käynnistämään välittömästi tutkinnan hankintayksikön (Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)) ja toimittajan (Istekki Oy, Y-tunnus 2292633-0) välisistä suorahankinnoista ja ketjutetuista alihankintasopimuksista (240.00 milj. EUR/v);</t>
+          <t>3. VAATIMUKSET KILPAILU- JA KULUTTAJAVIRASTOLLE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3542,7 +3871,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2) Esittämään markkinaoikeudelle hankintalain 156 §:n mukaisen TEHOTTOMUUSSEURAAMUKSEN määräämistä lainvastaisille suorahankintasopimuksille;</t>
+          <t>Pyydämme Kilpailu- ja kuluttajavirastoa hankintalain 139–141 §:n nojalla:</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3584,40 +3913,1792 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>1) Käynnistämään välittömästi tutkinnan hankintayksikön (Vähemmistöomistaja-HVA:t &amp; &gt;150 kuntaa (pääomistajat Pirha &amp; Pshyva)) ja toimittajan (Istekki Oy, Y-tunnus 2292633-0) välisistä suorahankinnoista ja ketjutetuista alihankintasopimuksista (240.00 milj. EUR/v);</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2) Esittämään markkinaoikeudelle hankintalain 156 §:n mukaisen TEHOTTOMUUSSEURAAMUKSEN määräämistä lainvastaisille suorahankintasopimuksille;</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>3) Esittämään markkinaoikeudelle hankintalain 158 §:n mukaisen SEURAAMUSMAKSUN määräämistä sekä sopimuskauden lyhentämistä siten, että palvelut avataan välittömästi avoimeen kilpailutukseen.</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>KAIKKI 43 SUURINTA JULKISTA OSTAJAA (21 HYVINVOINTIALUETTA + HUS + 21 SUURINTA KAUPUNKIA)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Julkisuuslain (621/1999) 13 § ja 16.3 § velvoittaa jokaisen viranomaisen luovuttamaan ostolaskudatan 14 vrk kuluessa.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="1">
+        <is>
+          <t>Julkinen hankintayksikkö</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="1">
+        <is>
+          <t>Tyyppi (HVA / HUS / Kunta)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="1">
+        <is>
+          <t>PRH Y-tunnus (Modulo-11)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="1">
+        <is>
+          <t>Virallinen kirjaamo-sähköposti</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="1">
+        <is>
+          <t>Ulkoiset ostot (M€/v)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="1">
+        <is>
+          <t>Julkaiseeko avoimen ostolaskudatan?</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="1">
+        <is>
+          <t>Keskeiset sidosyksikkö- ja in-house-yhtiöt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HUS-yhtymä</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HUS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1567535-0</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>kirjaamo@hus.fi</t>
+        </is>
+      </c>
+      <c r="E4" s="2">
+        <v>1480.0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Oy Apotti Ab, Valtori</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pirkanmaan hyvinvointialue (Pirha)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3221308-6</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>kirjaamo@pirha.fi</t>
+        </is>
+      </c>
+      <c r="E5" s="2">
+        <v>1320.0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Istekki Oy, Fimlab Oy, Tuomi Logistiikka Oy, Monetra</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Varsinais-Suomen hyvinvointialue (Varha)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>3221065-1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>kirjaamo@varha.fi</t>
+        </is>
+      </c>
+      <c r="E6" s="2">
+        <v>1190.0</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Numera/Sarastia, Kaarea Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pohjois-Pohjanmaan hyvinvointialue (Pohde)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>3221326-2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>kirjaamo@pohde.fi</t>
+        </is>
+      </c>
+      <c r="E7" s="2">
+        <v>1080.0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Monetra Oy, Istekki Oy, Esko Systems Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Länsi-Uudenmaan hyvinvointialue (Luvn)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3221347-3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>kirjaamo@luvn.fi</t>
+        </is>
+      </c>
+      <c r="E8" s="2">
+        <v>1040.0</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Numera/Sarastia, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Vantaan ja Keravan hyvinvointialue (Vake)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>3221356-1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>kirjaamo@vakehyva.fi</t>
+        </is>
+      </c>
+      <c r="E9" s="2">
+        <v>790.0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Oy Apotti Ab, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Keski-Suomen hyvinvointialue (Hyvaks)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3221318-2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>kirjaamo@hyvaks.fi</t>
+        </is>
+      </c>
+      <c r="E10" s="2">
+        <v>690.0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Istekki Oy, Monetra Oy, 2M-IT Oy, Fimlab Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Pohjois-Savon hyvinvointialue (Pshyva)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3221316-6</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>kirjaamo@pshyva.fi</t>
+        </is>
+      </c>
+      <c r="E11" s="2">
+        <v>660.0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Istekki Oy, ISLAB, Sansia Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Satakunnan hyvinvointialue (Sata)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>3221302-7</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>kirjaamo@sata.fi</t>
+        </is>
+      </c>
+      <c r="E12" s="2">
+        <v>610.0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Päijät-Hämeen hyvinvointialue (Päijät-Sote)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>3221309-4</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>kirjaamo@paijatha.fi</t>
+        </is>
+      </c>
+      <c r="E13" s="2">
+        <v>590.0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Fimlab Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Lapin hyvinvointialue (Lapha)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>3221332-6</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>kirjaamo@lapha.fi</t>
+        </is>
+      </c>
+      <c r="E14" s="2">
+        <v>580.0</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Numera/Sarastia, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Keski-Uudenmaan hyvinvointialue (Keusote)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>3221346-5</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>kirjaamo@keusote.fi</t>
+        </is>
+      </c>
+      <c r="E15" s="2">
+        <v>540.0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Numera/Sarastia, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Kanta-Hämeen hyvinvointialue (Oma Häme)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>3221307-8</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>kirjaamo@omahame.fi</t>
+        </is>
+      </c>
+      <c r="E16" s="2">
+        <v>495.0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Numera/Sarastia, Fimlab Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Etelä-Pohjanmaan hyvinvointialue (Hyvaep)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>3221323-8</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>kirjaamo@hyvaep.fi</t>
+        </is>
+      </c>
+      <c r="E17" s="2">
+        <v>490.0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Istekki Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Kymenlaakson hyvinvointialue (Kymenhva)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>3221311-5</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>kirjaamo@kymenhva.fi</t>
+        </is>
+      </c>
+      <c r="E18" s="2">
+        <v>480.0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Meita Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Pohjois-Karjalan hyvinvointialue (Siun sote)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>3221317-4</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>kirjaamo@siunsote.fi</t>
+        </is>
+      </c>
+      <c r="E19" s="2">
+        <v>460.0</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Istekki Oy, Polkka Oy, ISLAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Pohjanmaan hyvinvointialue (Österbotten)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>3221324-6</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>kirjaamo@ovph.fi</t>
+        </is>
+      </c>
+      <c r="E20" s="2">
+        <v>440.0</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Fimlab Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Etelä-Savon hyvinvointialue (Eloisa)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>3221315-8</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>kirjaamo@etelasavonha.fi</t>
+        </is>
+      </c>
+      <c r="E21" s="2">
+        <v>410.0</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Istekki Oy, Meita Oy, ISLAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Etelä-Karjalan hyvinvointialue (Ekhva)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>3221313-1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>kirjaamo@ekhva.fi</t>
+        </is>
+      </c>
+      <c r="E22" s="2">
+        <v>385.0</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Meita Oy, 2M-IT Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Itä-Uudenmaan hyvinvointialue (Itä-Uusimaa)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>3221339-3</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>kirjaamo@itauusimaa.fi</t>
+        </is>
+      </c>
+      <c r="E23" s="2">
+        <v>275.0</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Numera/Sarastia, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Kainuun hyvinvointialue (Kainuu)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>3221331-8</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>kirjaamo@kainuu.fi</t>
+        </is>
+      </c>
+      <c r="E24" s="2">
+        <v>250.0</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Istekki Oy, Monetra Oy, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Keski-Pohjanmaan hyvinvointialue (Soite)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HVA</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>3221325-4</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>kirjaamo@soite.fi</t>
+        </is>
+      </c>
+      <c r="E25" s="2">
+        <v>235.0</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2M-IT Oy, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Helsingin kaupunki</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>0201256-6</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>helsinki.kirjaamo@hel.fi</t>
+        </is>
+      </c>
+      <c r="E26" s="2">
+        <v>2450.0</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Oy Apotti Ab, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Espoon kaupunki</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>0101263-6</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>kirjaamo@espoo.fi</t>
+        </is>
+      </c>
+      <c r="E27" s="2">
+        <v>1120.0</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Tiera Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Tampereen kaupunki</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0211675-2</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>kirjaamo@tampere.fi</t>
+        </is>
+      </c>
+      <c r="E28" s="2">
+        <v>980.0</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Monetra Pirkanmaa, Istekki Oy, Tuomi Logistiikka Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Vantaan kaupunki</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0124610-9</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>kirjaamo@vantaa.fi</t>
+        </is>
+      </c>
+      <c r="E29" s="2">
+        <v>890.0</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Tiera Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Oulun kaupunki</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0187690-1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>kirjaamo@ouka.fi</t>
+        </is>
+      </c>
+      <c r="E30" s="2">
+        <v>740.0</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Monetra Oulu Oy, Istekki Oy, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Turun kaupunki</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>0204819-8</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>kirjaamo@turku.fi</t>
+        </is>
+      </c>
+      <c r="E31" s="2">
+        <v>720.0</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Kaarea Oy, Tiera Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Jyväskylän kaupunki</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>0174666-4</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>kirjaamo@jyvaskyla.fi</t>
+        </is>
+      </c>
+      <c r="E32" s="2">
+        <v>480.0</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Monetra Keski-Suomi Oy, Istekki Oy, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Kuopion kaupunki</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>0171450-7</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>kirjaamo@kuopio.fi</t>
+        </is>
+      </c>
+      <c r="E33" s="2">
+        <v>430.0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Istekki Oy, Sansia Oy, Monetra Pohjois-Savo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Lahden kaupunki</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>0149669-3</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>kirjaamo@lahti.fi</t>
+        </is>
+      </c>
+      <c r="E34" s="2">
+        <v>410.0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Tiera Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Porin kaupunki</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>0137323-9</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>kirjaamo@pori.fi</t>
+        </is>
+      </c>
+      <c r="E35" s="2">
+        <v>310.0</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Numera/Sarastia, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Kouvolan kaupunki</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>0161075-9</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>kirjaamo@kouvola.fi</t>
+        </is>
+      </c>
+      <c r="E36" s="2">
+        <v>295.0</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Meita Oy, Tiera Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Joensuun kaupunki</t>
+        </is>
+      </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t/>
+          <t>Kunta</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t/>
+          <t>0242746-2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>kirjaamo@joensuu.fi</t>
+        </is>
+      </c>
+      <c r="E37" s="2">
+        <v>270.0</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t/>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
+          <t>Polkka Oy, Tiera Oy, Meita Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Lappeenrannan kaupunki</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>0162193-3</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>kirjaamo@lappeenranta.fi</t>
+        </is>
+      </c>
+      <c r="E38" s="2">
+        <v>265.0</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Meita Oy, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Hämeenlinnan kaupunki</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>0146921-4</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>hameenlinnan.kaupunki@hameenlinna.fi</t>
+        </is>
+      </c>
+      <c r="E39" s="2">
+        <v>245.0</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>KYLLÄ</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Numera/Sarastia, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Vaasan kaupunki</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>0209602-6</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>kirjaamo@vaasa.fi</t>
+        </is>
+      </c>
+      <c r="E40" s="2">
+        <v>240.0</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Tiera Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Seinäjoen kaupunki</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1928736-3</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>kirjaamo@seinajoki.fi</t>
+        </is>
+      </c>
+      <c r="E41" s="2">
+        <v>225.0</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Tiera Oy, Istekki Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Rovaniemen kaupunki</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1978283-1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>kirjaamo@rovaniemi.fi</t>
+        </is>
+      </c>
+      <c r="E42" s="2">
+        <v>215.0</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Tiera Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Mikkelin kaupunki</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>0165116-3</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>kirjaamo@mikkeli.fi</t>
+        </is>
+      </c>
+      <c r="E43" s="2">
+        <v>195.0</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Meita Oy, Tiera Oy, Istekki Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Kotkan kaupunki</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>0161077-5</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>kirjaamo@kotka.fi</t>
+        </is>
+      </c>
+      <c r="E44" s="2">
+        <v>190.0</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Meita Oy, Tiera Oy</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Salon kaupunki</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>0139533-1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>kirjaamo@salo.fi</t>
+        </is>
+      </c>
+      <c r="E45" s="2">
+        <v>175.0</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Tiera Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Porvoon kaupunki</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Kunta</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1061512-1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>kirjaamo@porvoo.fi</t>
+        </is>
+      </c>
+      <c r="E46" s="2">
+        <v>170.0</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>EI (Vaadi JulkL 13 § tietopyynnöllä)</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Tiera Oy, Numera/Sarastia</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>YHTEENSÄ (43 JULKISTA HANKINTAYKSIKKÖÄ)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E47" s="2">
+        <f>SUM(E4:E46)</f>
+        <v>25505.0</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
Remediate GPT-6 Astra & Claude Opus 5.5 Red Team findings: calibrate Apotti HUS/Helsinki/Vake 147.7M split, branch inhouse modals/KKV filings on >=10% equity, unify 832.63M/yr totals & neutralize Excel tabs
</commit_message>
<xml_diff>
--- a/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
+++ b/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="01_Yhteenveto_Leikkuri" sheetId="1" r:id="rId1"/>
-    <sheet name="02_Sidosyksikko_Kartellit" sheetId="2" r:id="rId2"/>
+    <sheet name="01_Yhteenveto_Tehokkuus" sheetId="1" r:id="rId1"/>
+    <sheet name="02_Sidosyksikot_15_Yksikkoa" sheetId="2" r:id="rId2"/>
     <sheet name="03_Alueiden_Hintavertailu_P25" sheetId="3" r:id="rId3"/>
-    <sheet name="04_MAO_Hilma_1Tarjous_Tapaukset" sheetId="4" r:id="rId4"/>
+    <sheet name="04_MAO_ja_KHO_Ratkaisut" sheetId="4" r:id="rId4"/>
     <sheet name="05_Kaikki_43_Julkista_Ostajaa" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
@@ -159,48 +159,64 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <v>2538.23</v>
+        <v>2521.68</v>
       </c>
       <c r="C5" s="2">
-        <v>2538.23</v>
+        <v>2521.68</v>
       </c>
       <c r="D5" s="2">
-        <v>594.4</v>
+        <v>582.71</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3. Yhden tarjouksen kilpailutusten (KKV: n. 15–16 % hankinnoista) ja suorahankintojen avaaminen kilpailulle</t>
+          <t>3. Dokumentoidut MAO- ja KHO-oikeustapaukset (10 Finlex/KKV-ratkaisua 2023–2025: suorahankinnat ja kilpailutukset)</t>
         </is>
       </c>
       <c r="B6" s="2">
-        <v>5800.0</v>
+        <v>78.61</v>
       </c>
       <c r="C6" s="2">
-        <v>1500.0</v>
+        <v>70.61</v>
       </c>
       <c r="D6" s="2">
-        <v>225.0</v>
+        <v>18.93</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>YHTEENSÄ (LASKENNALLINEN RAKENTEELLINEN SÄÄSTÖPOTENTIAALI, M€/V)</t>
+          <t>YHTEENSÄ (SUORAAN MALLINNETUT AINEISTOT, M€/V)</t>
         </is>
       </c>
       <c r="B7" s="2">
         <f>SUM(B4:B6)</f>
-        <v>10301.63</v>
+        <v>4563.69</v>
       </c>
       <c r="C7" s="2">
         <f>SUM(C4:C6)</f>
-        <v>5292.93</v>
+        <v>3846.99</v>
       </c>
       <c r="D7" s="2">
         <f>SUM(D4:D6)</f>
-        <v>1050.39</v>
+        <v>832.63</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kansallinen makropotentiaali koko 38 700 M€/v hankintakannassa (sis. KKV ~1 500 M€/v yhden tarjouksen kilpailutukset)</t>
+        </is>
+      </c>
+      <c r="B8" s="2">
+        <v>38700.0</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1100.0</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2200.0</v>
       </c>
     </row>
   </sheetData>
@@ -1026,7 +1042,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>YHTEENSÄ (15 SIDOSYKSIKKÖJÄTTIÄ)</t>
+          <t>YHTEENSÄ (15 SIDOSYKSIKKÖÄ JA PALVELUKESKUSTA)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1938,7 +1954,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Vake (Apotti-kokonaiskustannus/käyttäjä)</t>
+          <t>Vake (Apotti-osuus 18,7 % — kustannus/käyttäjä)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1975,7 +1991,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HUS-yhtymä (Apotti-kokonaiskustannus/käyttäjä)</t>
+          <t>HUS &amp; Helsingin sote (Apotti-osuus 81,3 % — kustannus/käyttäjä)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1989,7 +2005,7 @@
         </is>
       </c>
       <c r="D24" s="2">
-        <v>22000.0</v>
+        <v>19330.0</v>
       </c>
       <c r="E24" s="2">
         <v>6200.0</v>
@@ -2002,11 +2018,11 @@
       </c>
       <c r="H24" s="2">
         <f>ROUND(D24*E24,2)</f>
-        <v>136400000.0</v>
+        <v>119846000.0</v>
       </c>
       <c r="I24" s="2">
         <f>ROUND(IF(E24&gt;F24,D24*(E24-F24),0),2)</f>
-        <v>96360000.0</v>
+        <v>84665400.0</v>
       </c>
     </row>
     <row r="25">
@@ -2454,11 +2470,11 @@
       </c>
       <c r="H36" s="2">
         <f>SUM(H4:H35)</f>
-        <v>2538230000.0</v>
+        <v>2521676000.0</v>
       </c>
       <c r="I36" s="2">
         <f>SUM(I4:I35)</f>
-        <v>594402000.0</v>
+        <v>582707400.0</v>
       </c>
     </row>
   </sheetData>
@@ -2481,7 +2497,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t>MARKKINAOIKEUS (MAO) &amp; HILMA 1–2 TARJOUKSEN KARTELLIHANKINNAT SEKÄ 0 € KKV-VALITUSPOHJAT</t>
+          <t>MARKKINAOIKEUDEN (MAO) JA KORKEIMMAN HALLINTO-OIKEUDEN (KHO) RATKAISUT (10 TAPAUSTA) SEKÄ 0 € HALLINTOPOHJAT</t>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
@@ -2523,7 +2539,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jokainen alle 2 tarjouksen sopimus &gt;100 000 € luokassa, jossa on &gt;=5 pk-haastajaa, merkitään uudelleenkilpailutettavaksi.</t>
+          <t>Vahvistetut Finlex / KKV -ratkaisut (2023–2025) sidosyksikköomistuksesta, suorahankinnoista ja tarjouskilpailuista.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2565,7 +2581,7 @@
     <row r="3">
       <c r="A3" t="inlineStr" s="1">
         <is>
-          <t>MAO / Hilma -tapaus</t>
+          <t>MAO / KHO -ratkaisu</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="1">
@@ -2590,17 +2606,17 @@
       </c>
       <c r="F3" t="inlineStr" s="1">
         <is>
-          <t>Kelpoiset PK-haastajat (kpl)</t>
+          <t>Kelpoiset PK-toimittajat (kpl)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr" s="1">
         <is>
-          <t>Kilpailunrajoitus / Lukitusmekanismi</t>
+          <t>Oikeustapauksen kuvaus (Finlex / KKV)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr" s="1">
         <is>
-          <t>Odotettu vuosisäästö (€/v)</t>
+          <t>Laskennallinen säästöpotentiaali (€/v)</t>
         </is>
       </c>
     </row>
@@ -2733,7 +2749,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KKV:n esitys: Kaupunki jatkoi matkailu- ja markkinointipalveluiden ostoja vanhan vuoden 2010 sopimuksen nojalla ilman kilpailutusta. Markkinaoikeus määräsi 40 000 € seuraamusmaksun.</t>
+          <t>KKV:n esitys: Kaupunki jatkoi matkailu- ja markkinointipalveluiden ostoja vanhan vuoden 2011 sopimuksen nojalla ilman kilpailutusta. Markkinaoikeus määräsi 40 000 € seuraamusmaksun.</t>
         </is>
       </c>
       <c r="H7" s="2">
@@ -3913,7 +3929,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1) Selvittämään, täyttävätkö pienosakkaiden (Pirha, Pshyva (pääomistajat) sekä kymmenet pienomistajakunnat ja -HVA:t (&lt;10 %)) suorahankinnat yksiköltä Istekki Oy (Y-tunnus 2292633-0) hankintalain 15 §:n ja KHO 8.10.2025 (taltio 2250) mukaiset edellytykset;</t>
+          <t>1) Selvittämään, täyttävätkö pienosakkaiden (Pirha, Pshyva (pääomistajat) sekä kymmenet pienomistajakunnat ja -HVA:t (&lt;10 %), viiteosuus 0.40 %) suorahankinnat yksiköltä Istekki Oy (Y-tunnus 2292633-0) hankintalain 15 §:n ja KHO 8.10.2025 (taltio 2250) mukaiset määräysvaltaedellytykset;</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3955,7 +3971,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2) Antamaan tarvittaessa hankintalain 140 §:n mukaisen huomautuksen tai ohjauksen avoimen kilpailutuksen järjestämisestä.</t>
+          <t>2) Antamaan tarvittaessa hankintalain 140 §:n mukaisen huomautuksen tai ohjauksen pienosakkaiden hankintojen saattamiseksi avoimen kilpailutuksen piiriin.</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4152,7 +4168,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Oy Apotti Ab, Valtori</t>
+          <t>Oy Apotti Ab, HUS Diagnostiikkakeskus / Hansel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Iteration 2 Red-Team Upgrade: 31-row P25 benchmark & 10-row MAO/KHO tables, CSV exports, dual KKV/Oikaisu switcher & PRH Y-tunnus lookup
</commit_message>
<xml_diff>
--- a/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
+++ b/dist/Sote_ja_Kunta_Kartelli_Matriisi_2026.xlsx
@@ -127,7 +127,7 @@
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t>Pienomistus / Vertailukanta (M€/v)</t>
+          <t>Hajautetun omistuksen (&lt;10 %) yhtiöt / Vertailukanta (M€/v)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="1">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="G3" t="inlineStr" s="1">
         <is>
-          <t>Ylihinta vs. P25 (%)</t>
+          <t>Ero vs. P25-vertailutaso (%)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr" s="1">

</xml_diff>